<commit_message>
Add BT profile select hold tap
</commit_message>
<xml_diff>
--- a/physical_layout.xlsx
+++ b/physical_layout.xlsx
@@ -9,11 +9,12 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="34725" windowHeight="16110" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="34725" windowHeight="16110" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
+    <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="152511"/>
   <extLst>
@@ -25,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="219" uniqueCount="91">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="214" uniqueCount="86">
   <si>
     <t>X</t>
     <phoneticPr fontId="1"/>
@@ -93,24 +94,6 @@
     <phoneticPr fontId="1"/>
   </si>
   <si>
-    <t xml:space="preserve">    physical_layout0: physical_layout_0 {</t>
-  </si>
-  <si>
-    <t xml:space="preserve">        compatible = "zmk,physical-layout";</t>
-  </si>
-  <si>
-    <t xml:space="preserve">        display-name = "Default Layout";</t>
-  </si>
-  <si>
-    <t xml:space="preserve">        transform = &lt;&amp;default_transform&gt;;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">        kscan = &lt;&amp;kscan_composite&gt;;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">        keys  //                     w   h   x  y   rot rx ry</t>
-  </si>
-  <si>
     <t xml:space="preserve">            =</t>
   </si>
   <si>
@@ -319,6 +302,9 @@
   </si>
   <si>
     <t xml:space="preserve">    };</t>
+  </si>
+  <si>
+    <t>&amp;none &amp;none &amp;none &amp;none &amp;trans &amp;none &amp;none &amp;trans &amp;none &amp;none &amp;none &amp;none &amp;none</t>
   </si>
 </sst>
 </file>
@@ -788,11 +774,11 @@
         <v>100</v>
       </c>
       <c r="J3">
-        <f t="shared" ref="J3:J57" si="0">D3+G3/2</f>
+        <f t="shared" ref="J3:J7" si="0">D3+G3/2</f>
         <v>150</v>
       </c>
       <c r="K3">
-        <f t="shared" ref="K3:K57" si="1">E3+H3/2</f>
+        <f t="shared" ref="K3:K7" si="1">E3+H3/2</f>
         <v>100</v>
       </c>
       <c r="L3">
@@ -806,7 +792,7 @@
         <v>12</v>
       </c>
       <c r="P3" t="str">
-        <f t="shared" ref="P3:P57" si="2">CONCATENATE("&lt;&amp;key_physical_attrs "&amp;G3&amp;" "&amp;H3&amp;" "&amp;J3&amp;" "&amp;K3&amp;" "&amp;J3&amp;" "&amp;K3&amp;" "&amp;L3&amp;" "&amp;"&gt;")</f>
+        <f t="shared" ref="P3:P7" si="2">CONCATENATE("&lt;&amp;key_physical_attrs "&amp;G3&amp;" "&amp;H3&amp;" "&amp;J3&amp;" "&amp;K3&amp;" "&amp;J3&amp;" "&amp;K3&amp;" "&amp;L3&amp;" "&amp;"&gt;")</f>
         <v>&lt;&amp;key_physical_attrs 100 100 150 100 150 100 0 &gt;</v>
       </c>
     </row>
@@ -815,7 +801,7 @@
         <v>3</v>
       </c>
       <c r="B4">
-        <f t="shared" ref="B4:B13" si="3">B3</f>
+        <f t="shared" ref="B4:B7" si="3">B3</f>
         <v>0</v>
       </c>
       <c r="C4">
@@ -845,7 +831,7 @@
         <v>0</v>
       </c>
       <c r="M4">
-        <f t="shared" ref="M4:M57" si="4">M3+1</f>
+        <f t="shared" ref="M4:M7" si="4">M3+1</f>
         <v>2</v>
       </c>
       <c r="O4" t="s">
@@ -1384,7 +1370,7 @@
         <v>100</v>
       </c>
       <c r="E17">
-        <f t="shared" ref="E17:E34" si="9">E3+100</f>
+        <f t="shared" ref="E17:E27" si="9">E3+100</f>
         <v>150</v>
       </c>
       <c r="G17">
@@ -3582,50 +3568,68 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B76"/>
+  <dimension ref="A1:B70"/>
   <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.15"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A1" t="s">
         <v>15</v>
       </c>
+      <c r="B1" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A2" t="s">
-        <v>16</v>
+        <v>17</v>
+      </c>
+      <c r="B2" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A3" t="s">
         <v>17</v>
       </c>
+      <c r="B3" t="s">
+        <v>19</v>
+      </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A4" t="s">
-        <v>18</v>
+        <v>17</v>
+      </c>
+      <c r="B4" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A5" t="s">
-        <v>19</v>
+        <v>17</v>
+      </c>
+      <c r="B5" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A6" t="s">
-        <v>20</v>
+        <v>17</v>
+      </c>
+      <c r="B6" t="s">
+        <v>22</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A7" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="B7" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A8" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="B8" t="s">
         <v>24</v>
@@ -3633,7 +3637,7 @@
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A9" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="B9" t="s">
         <v>25</v>
@@ -3641,7 +3645,7 @@
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A10" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="B10" t="s">
         <v>26</v>
@@ -3649,7 +3653,7 @@
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A11" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="B11" t="s">
         <v>27</v>
@@ -3657,7 +3661,7 @@
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A12" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="B12" t="s">
         <v>28</v>
@@ -3665,7 +3669,7 @@
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A13" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="B13" t="s">
         <v>29</v>
@@ -3673,7 +3677,7 @@
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A14" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="B14" t="s">
         <v>30</v>
@@ -3681,7 +3685,7 @@
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A15" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="B15" t="s">
         <v>31</v>
@@ -3689,7 +3693,7 @@
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A16" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="B16" t="s">
         <v>32</v>
@@ -3697,7 +3701,7 @@
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A17" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="B17" t="s">
         <v>33</v>
@@ -3705,7 +3709,7 @@
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A18" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="B18" t="s">
         <v>34</v>
@@ -3713,7 +3717,7 @@
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A19" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="B19" t="s">
         <v>35</v>
@@ -3721,7 +3725,7 @@
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A20" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="B20" t="s">
         <v>36</v>
@@ -3729,7 +3733,7 @@
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A21" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="B21" t="s">
         <v>37</v>
@@ -3737,7 +3741,7 @@
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A22" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="B22" t="s">
         <v>38</v>
@@ -3745,7 +3749,7 @@
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A23" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="B23" t="s">
         <v>39</v>
@@ -3753,7 +3757,7 @@
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A24" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="B24" t="s">
         <v>40</v>
@@ -3761,7 +3765,7 @@
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A25" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="B25" t="s">
         <v>41</v>
@@ -3769,7 +3773,7 @@
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A26" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="B26" t="s">
         <v>42</v>
@@ -3777,7 +3781,7 @@
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A27" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="B27" t="s">
         <v>43</v>
@@ -3785,7 +3789,7 @@
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A28" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="B28" t="s">
         <v>44</v>
@@ -3793,7 +3797,7 @@
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A29" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="B29" t="s">
         <v>45</v>
@@ -3801,7 +3805,7 @@
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A30" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="B30" t="s">
         <v>46</v>
@@ -3809,7 +3813,7 @@
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A31" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="B31" t="s">
         <v>47</v>
@@ -3817,7 +3821,7 @@
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A32" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="B32" t="s">
         <v>48</v>
@@ -3825,7 +3829,7 @@
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A33" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="B33" t="s">
         <v>49</v>
@@ -3833,7 +3837,7 @@
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A34" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="B34" t="s">
         <v>50</v>
@@ -3841,7 +3845,7 @@
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A35" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="B35" t="s">
         <v>51</v>
@@ -3849,7 +3853,7 @@
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A36" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="B36" t="s">
         <v>52</v>
@@ -3857,7 +3861,7 @@
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A37" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="B37" t="s">
         <v>53</v>
@@ -3865,7 +3869,7 @@
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A38" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="B38" t="s">
         <v>54</v>
@@ -3873,7 +3877,7 @@
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A39" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="B39" t="s">
         <v>55</v>
@@ -3881,7 +3885,7 @@
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A40" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="B40" t="s">
         <v>56</v>
@@ -3889,7 +3893,7 @@
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A41" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="B41" t="s">
         <v>57</v>
@@ -3897,7 +3901,7 @@
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A42" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="B42" t="s">
         <v>58</v>
@@ -3905,7 +3909,7 @@
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A43" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="B43" t="s">
         <v>59</v>
@@ -3913,7 +3917,7 @@
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A44" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="B44" t="s">
         <v>60</v>
@@ -3921,7 +3925,7 @@
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A45" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="B45" t="s">
         <v>61</v>
@@ -3929,7 +3933,7 @@
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A46" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="B46" t="s">
         <v>62</v>
@@ -3937,7 +3941,7 @@
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A47" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="B47" t="s">
         <v>63</v>
@@ -3945,7 +3949,7 @@
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A48" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="B48" t="s">
         <v>64</v>
@@ -3953,7 +3957,7 @@
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A49" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="B49" t="s">
         <v>65</v>
@@ -3961,7 +3965,7 @@
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A50" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="B50" t="s">
         <v>66</v>
@@ -3969,7 +3973,7 @@
     </row>
     <row r="51" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A51" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="B51" t="s">
         <v>67</v>
@@ -3977,7 +3981,7 @@
     </row>
     <row r="52" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A52" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="B52" t="s">
         <v>68</v>
@@ -3985,7 +3989,7 @@
     </row>
     <row r="53" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A53" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="B53" t="s">
         <v>69</v>
@@ -3993,7 +3997,7 @@
     </row>
     <row r="54" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A54" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="B54" t="s">
         <v>70</v>
@@ -4001,7 +4005,7 @@
     </row>
     <row r="55" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A55" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="B55" t="s">
         <v>71</v>
@@ -4009,7 +4013,7 @@
     </row>
     <row r="56" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A56" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="B56" t="s">
         <v>72</v>
@@ -4017,7 +4021,7 @@
     </row>
     <row r="57" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A57" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="B57" t="s">
         <v>73</v>
@@ -4025,7 +4029,7 @@
     </row>
     <row r="58" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A58" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="B58" t="s">
         <v>74</v>
@@ -4033,7 +4037,7 @@
     </row>
     <row r="59" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A59" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="B59" t="s">
         <v>75</v>
@@ -4041,7 +4045,7 @@
     </row>
     <row r="60" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A60" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="B60" t="s">
         <v>76</v>
@@ -4049,7 +4053,7 @@
     </row>
     <row r="61" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A61" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="B61" t="s">
         <v>77</v>
@@ -4057,7 +4061,7 @@
     </row>
     <row r="62" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A62" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="B62" t="s">
         <v>78</v>
@@ -4065,7 +4069,7 @@
     </row>
     <row r="63" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A63" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="B63" t="s">
         <v>79</v>
@@ -4073,7 +4077,7 @@
     </row>
     <row r="64" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A64" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="B64" t="s">
         <v>80</v>
@@ -4081,7 +4085,7 @@
     </row>
     <row r="65" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A65" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="B65" t="s">
         <v>81</v>
@@ -4089,7 +4093,7 @@
     </row>
     <row r="66" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A66" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="B66" t="s">
         <v>82</v>
@@ -4097,60 +4101,28 @@
     </row>
     <row r="67" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A67" t="s">
-        <v>23</v>
-      </c>
-      <c r="B67" t="s">
         <v>83</v>
-      </c>
-    </row>
-    <row r="68" spans="1:2" x14ac:dyDescent="0.15">
-      <c r="A68" t="s">
-        <v>23</v>
-      </c>
-      <c r="B68" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="69" spans="1:2" x14ac:dyDescent="0.15">
-      <c r="A69" t="s">
-        <v>23</v>
-      </c>
-      <c r="B69" t="s">
-        <v>85</v>
       </c>
     </row>
     <row r="70" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A70" t="s">
-        <v>23</v>
-      </c>
-      <c r="B70" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="71" spans="1:2" x14ac:dyDescent="0.15">
-      <c r="A71" t="s">
-        <v>23</v>
-      </c>
-      <c r="B71" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="72" spans="1:2" x14ac:dyDescent="0.15">
-      <c r="A72" t="s">
-        <v>23</v>
-      </c>
-      <c r="B72" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="73" spans="1:2" x14ac:dyDescent="0.15">
-      <c r="A73" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="76" spans="1:2" x14ac:dyDescent="0.15">
-      <c r="A76" t="s">
-        <v>90</v>
+        <v>84</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.15"/>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.15">
+      <c r="A1" t="s">
+        <v>85</v>
       </c>
     </row>
   </sheetData>

</xml_diff>